<commit_message>
Creación de Informe de pruebas API
</commit_message>
<xml_diff>
--- a/api_testing/casos_api.xlsx
+++ b/api_testing/casos_api.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brenr\OneDrive\Desktop\Bren\ADA\QA TESTING\ProyectoFinal-Ruejas\api_testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3C50C96-0BAE-4FCF-86D0-088CC68E2F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEFCCD0E-B819-4EBF-A316-ED104124AC7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -156,9 +156,6 @@
     <t>API-10</t>
   </si>
   <si>
-    <t>/cars</t>
-  </si>
-  <si>
     <t xml:space="preserve">Obtener carritos </t>
   </si>
   <si>
@@ -172,6 +169,9 @@
   </si>
   <si>
     <t>200 OK e imagen del producto</t>
+  </si>
+  <si>
+    <t>/carts</t>
   </si>
 </sst>
 </file>
@@ -704,10 +704,10 @@
         <v>6</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>44</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>31</v>
@@ -715,19 +715,19 @@
     </row>
     <row r="12" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C12" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agregué detalles finales para el cierre del proyecto y su posterior evaluación
</commit_message>
<xml_diff>
--- a/api_testing/casos_api.xlsx
+++ b/api_testing/casos_api.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brenr\OneDrive\Desktop\Bren\ADA\QA TESTING\ProyectoFinal-Ruejas\api_testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEFCCD0E-B819-4EBF-A316-ED104124AC7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7AE7753-0860-4D0E-9EA9-393307D8478E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="51">
   <si>
     <t>ID</t>
   </si>
@@ -172,6 +172,12 @@
   </si>
   <si>
     <t>/carts</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>PASS</t>
   </si>
 </sst>
 </file>
@@ -240,7 +246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -257,6 +263,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -518,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.5546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="62" customWidth="1"/>
@@ -526,7 +533,7 @@
     <col min="5" max="5" width="57.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -542,8 +549,11 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F1" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -559,8 +569,11 @@
       <c r="E2" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F2" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -576,8 +589,11 @@
       <c r="E3" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F3" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
@@ -593,8 +609,11 @@
       <c r="E4" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F4" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -610,8 +629,11 @@
       <c r="E5" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="F5" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -627,8 +649,11 @@
       <c r="E6" s="4" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="F6" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>28</v>
       </c>
@@ -644,8 +669,11 @@
       <c r="E7" s="4" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="F7" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>32</v>
       </c>
@@ -661,8 +689,11 @@
       <c r="E8" s="4" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F8" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>36</v>
       </c>
@@ -678,8 +709,11 @@
       <c r="E9" s="4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="F9" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>39</v>
       </c>
@@ -695,8 +729,11 @@
       <c r="E10" s="4" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="F10" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>42</v>
       </c>
@@ -712,8 +749,11 @@
       <c r="E11" s="4" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F11" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>44</v>
       </c>
@@ -728,6 +768,9 @@
       </c>
       <c r="E12" s="4" t="s">
         <v>47</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>